<commit_message>
update ap cost rule and hp commonality rule / fix typo
</commit_message>
<xml_diff>
--- a/Data/Monster.xlsx
+++ b/Data/Monster.xlsx
@@ -1,14 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CombatCalculatorTest\Data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394EE9FF-9738-469C-886F-B14E816B318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="MonsterIndex" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="MonsterBaseStat" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="MonsterSkill" sheetId="3" r:id="rId6"/>
+    <sheet name="MonsterIndex" sheetId="1" r:id="rId1"/>
+    <sheet name="MonsterBaseStat" sheetId="2" r:id="rId2"/>
+    <sheet name="MonsterSkill" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -24,18 +33,9 @@
     <t>MonsterWeight</t>
   </si>
   <si>
-    <t>Monste01</t>
-  </si>
-  <si>
     <t>Normal</t>
   </si>
   <si>
-    <t>Monste02</t>
-  </si>
-  <si>
-    <t>Monste03</t>
-  </si>
-  <si>
     <t>Level</t>
   </si>
   <si>
@@ -75,9 +75,6 @@
     <t>Target</t>
   </si>
   <si>
-    <t>Monste01_1</t>
-  </si>
-  <si>
     <t>AfterEnemyAttackPhase</t>
   </si>
   <si>
@@ -93,40 +90,72 @@
     <t>Player</t>
   </si>
   <si>
-    <t>Monste02_1</t>
-  </si>
-  <si>
-    <t>Monste03_1</t>
-  </si>
-  <si>
     <t>AddShield</t>
   </si>
   <si>
     <t>Self</t>
   </si>
   <si>
-    <t>Monste03_2</t>
+    <t>Monster01</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster02</t>
+  </si>
+  <si>
+    <t>Monster03</t>
+  </si>
+  <si>
+    <t>Monster01_1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster02_1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster03_1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster03_2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -134,7 +163,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -144,54 +173,52 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -381,17 +408,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -402,297 +432,302 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" s="4">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="4">
         <v>5</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="4">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="4">
-        <v>10.0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>24</v>
       </c>
       <c r="B2" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C2" s="4">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="D2" s="4">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="E2" s="4">
-        <v>300.0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="B3" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C3" s="4">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="D3" s="4">
-        <v>50.0</v>
+        <v>50</v>
       </c>
       <c r="E3" s="4">
-        <v>500.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>26</v>
       </c>
       <c r="B4" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="4">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="D4" s="4">
-        <v>100.0</v>
+        <v>100</v>
       </c>
       <c r="E4" s="4">
-        <v>1000.0</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="6" max="6" width="19.0"/>
-    <col customWidth="1" min="8" max="8" width="15.63"/>
-    <col customWidth="1" min="9" max="9" width="19.0"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" customWidth="1"/>
+    <col min="9" max="9" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="5">
+        <v>100</v>
+      </c>
+      <c r="E2" s="5">
+        <v>3</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="G2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="H2" s="5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="J2" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="5">
+        <v>100</v>
+      </c>
+      <c r="E3" s="5">
         <v>3</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="6">
-        <v>100.0</v>
-      </c>
-      <c r="E2" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="F2" s="6" t="s">
+      <c r="F3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="3" t="s">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="D4" s="6">
+        <v>10</v>
+      </c>
+      <c r="E4" s="5">
+        <v>5</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="6">
-        <v>100.0</v>
-      </c>
-      <c r="E3" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="F3" s="6" t="s">
+      <c r="D5" s="5">
+        <v>100</v>
+      </c>
+      <c r="E5" s="5">
+        <v>3</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="7">
-        <v>10.0</v>
-      </c>
-      <c r="E4" s="6">
-        <v>5.0</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="6">
-        <v>100.0</v>
-      </c>
-      <c r="E5" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>25</v>
-      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor log output: structured events, level filtering, noise reduction
- battle_reporter: replace regex-based metric extraction with direct payload key lookup; remove import re; fix auto_filter None check to prevent Excel repair warning
- battle_simulator: carry metrics in **extra payload instead of embedding in message strings; split ambiguous event_types (Apply→ApplyDamageMul/ApplyHealMul, OnEnemyAttack→AfterAttack); add _event() level param with _LEVEL_ORDER; mark EnemyCounter Tick as TRACE-only; suppress ApplyDamageMul/ApplyHealMul when multiplier=1.0
- Data/Monster.xlsx: adjust Monster03 stats

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Monster.xlsx
+++ b/Data/Monster.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CombatCalculatorTest\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394EE9FF-9738-469C-886F-B14E816B318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF7635FE-43F1-45E9-9B8C-E3D3B6A62BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -137,11 +137,13 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -705,7 +707,7 @@
         <v>5</v>
       </c>
       <c r="D5" s="5">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="E5" s="5">
         <v>3</v>

</xml_diff>